<commit_message>
Update proteomics analyses and pathway outputs
Sync the ten local Script folders, reorganize multi-factor ORA outputs, and retain the corrected C-vs-P GSEA result with one negative GO CC term and no C-vs-P Reactome terms.
</commit_message>
<xml_diff>
--- a/Script_5_single_factor_pathway/age_vs_young_GSEA/GSEA_summary_aged_vs_young_single_factor.xlsx
+++ b/Script_5_single_factor_pathway/age_vs_young_GSEA/GSEA_summary_aged_vs_young_single_factor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/outobi/Downloads/final analysis/final code/Script_5_single_factor_pathway/age_vs_young_GSEA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07336883-B9EA-CE41-9FE9-0E74EA107D4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4229803F-6F27-8041-95BB-689803A3DE82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10340" yWindow="5800" windowWidth="23260" windowHeight="13900" xr2:uid="{0CF324BB-1E02-42B0-A0C9-68BA90AF1E46}"/>
+    <workbookView xWindow="40980" yWindow="4840" windowWidth="23260" windowHeight="13900" xr2:uid="{0CF324BB-1E02-42B0-A0C9-68BA90AF1E46}"/>
   </bookViews>
   <sheets>
     <sheet name="GO aged" sheetId="6" r:id="rId1"/>
@@ -949,6 +949,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">

</xml_diff>